<commit_message>
unmatched witholding taxes for same year too
</commit_message>
<xml_diff>
--- a/tax_forms_template.xlsx
+++ b/tax_forms_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob\Downloads\‏‏‏‏‏‏‏‏tax_forms_generator - עותק - עותק - עותק\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob\OneDrive\Documents\Scripts\GitHub\IBKR1325\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36683EC5-59FB-4C33-A355-4991858AC87F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17F84BB-04E9-4D31-9D4A-F4DEBBCE7BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dividends" sheetId="6" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="51">
   <si>
     <t>במקום טופס 1325 - נספח ג(1)</t>
   </si>
@@ -176,9 +176,6 @@
   </si>
   <si>
     <t>שער מטח</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> לוודא שאין החזרי מס על דיבידנדים בשנה שלפני שמוסו במקור אבל ארה"ב לא היו אמורים לגבות אז החזירו בחזרה </t>
   </si>
   <si>
     <t xml:space="preserve">רווח הון (מט"ח) </t>
@@ -1635,9 +1632,7 @@
       <c r="AB1" s="5"/>
     </row>
     <row r="2" spans="1:28" ht="17.649999999999999">
-      <c r="D2" s="50" t="s">
-        <v>39</v>
-      </c>
+      <c r="D2" s="50"/>
       <c r="E2" s="13"/>
       <c r="F2" s="21"/>
       <c r="G2" s="4"/>
@@ -4414,7 +4409,7 @@
       <c r="U3" s="35"/>
       <c r="V3" s="35"/>
       <c r="W3" s="66" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="X3" s="65"/>
     </row>
@@ -4481,13 +4476,13 @@
         <v>28</v>
       </c>
       <c r="W4" s="36" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="X4" s="36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Y4" s="36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Z4"/>
     </row>
@@ -57838,10 +57833,10 @@
         <v>28</v>
       </c>
       <c r="W4" s="36" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="X4" s="36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Y4" s="37" t="s">
         <v>38</v>
@@ -61044,7 +61039,7 @@
     </row>
     <row r="2" spans="2:12" ht="15.75" customHeight="1">
       <c r="B2" s="69" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C2" s="69"/>
       <c r="D2" s="69"/>
@@ -61072,7 +61067,7 @@
     </row>
     <row r="4" spans="2:12" ht="17.649999999999999">
       <c r="B4" s="26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -61092,22 +61087,22 @@
         <v>21</v>
       </c>
       <c r="D5" s="59" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E5" s="59" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F5" s="59" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="60" t="s">
+      <c r="H5" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="61" t="s">
+      <c r="I5" s="62" t="s">
         <v>46</v>
-      </c>
-      <c r="I5" s="62" t="s">
-        <v>47</v>
       </c>
       <c r="K5" s="8"/>
     </row>

</xml_diff>

<commit_message>
Added Code for 1325
</commit_message>
<xml_diff>
--- a/tax_forms_template.xlsx
+++ b/tax_forms_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacob\OneDrive\Documents\Scripts\GitHub\IBKR1325\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1168F2E-D6F6-4E8C-82FD-48F5F037F489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2925829B-7090-4FA9-AC18-6E7E71416C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -211,7 +211,7 @@
     <t>עמלת פתיחת עסקה (מט"ח)</t>
   </si>
   <si>
-    <t>עמלות משנים עברו לא נמצאים בדוח ויחושבו כ0 משפיע על מכירות בשורט כי הערך שם יחושב עם העמלה(ממש שולי)</t>
+    <t xml:space="preserve">בעסקאות שורט שנפתחו בשנים קודמות הערך יופיע 0 כי אין מידע עליו בדוח הנתון הזה ישפיע על סכום מכירות שיחושב עם העמלה(הפרש שולי) </t>
   </si>
 </sst>
 </file>

</xml_diff>